<commit_message>
Add Lesson 4 basic spreadsheet functions
</commit_message>
<xml_diff>
--- a/02-excel/01-spreadsheet-fundamentals/excelSheet/Sales-data-practice.xlsx
+++ b/02-excel/01-spreadsheet-fundamentals/excelSheet/Sales-data-practice.xlsx
@@ -9,10 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sales Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Lesson 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
   <si>
     <t>Product</t>
   </si>
@@ -48,14 +50,79 @@
   </si>
   <si>
     <t>Water bottle</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Quantity Sold</t>
+  </si>
+  <si>
+    <t>Price per Unit</t>
+  </si>
+  <si>
+    <t>Sale Date</t>
+  </si>
+  <si>
+    <t>Laptop</t>
+  </si>
+  <si>
+    <t>Electronics</t>
+  </si>
+  <si>
+    <t>Mouse</t>
+  </si>
+  <si>
+    <t>Accessories</t>
+  </si>
+  <si>
+    <t>Keyboard</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>Headphone</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>(=C2*D2)</t>
+  </si>
+  <si>
+    <t>School Bag</t>
+  </si>
+  <si>
+    <t>Total Sales</t>
+  </si>
+  <si>
+    <t>(=SUM(D2:D4))</t>
+  </si>
+  <si>
+    <t>(=AVERAGE(D2:D4))</t>
+  </si>
+  <si>
+    <t>(=MIN(D2:D4))</t>
+  </si>
+  <si>
+    <t>(=MAX(D2:D4))</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -83,8 +150,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -442,4 +522,274 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="e">
+        <f>A1+B1</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>45000</v>
+      </c>
+      <c r="E2" s="5">
+        <v>46296</v>
+      </c>
+      <c r="F2">
+        <f>C2*D2</f>
+        <v>90000</v>
+      </c>
+      <c r="H2">
+        <v>100</v>
+      </c>
+      <c r="I2">
+        <v>20</v>
+      </c>
+      <c r="J2">
+        <f>H2/I2</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3">
+        <v>100</v>
+      </c>
+      <c r="D3">
+        <v>500</v>
+      </c>
+      <c r="E3" s="5">
+        <v>46297</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F6" si="0">C3*D3</f>
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>1200</v>
+      </c>
+      <c r="E4" s="5">
+        <v>46298</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>12000</v>
+      </c>
+      <c r="E5" s="5">
+        <v>46299</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>8</v>
+      </c>
+      <c r="D6">
+        <v>2000</v>
+      </c>
+      <c r="E6" s="5">
+        <v>46300</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2">
+        <v>50</v>
+      </c>
+      <c r="D2">
+        <f>B2*C2</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2">
+        <v>25</v>
+      </c>
+      <c r="C3" s="2">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <f t="shared" ref="D3:D4" si="0">B3*C3</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="2">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2">
+        <v>800</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <f>SUM(D2:D4)</f>
+        <v>3250</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <f>AVERAGE(D2:D4)</f>
+        <v>1083.3333333333333</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <f>MIN(D2:D4)</f>
+        <v>250</v>
+      </c>
+      <c r="E7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <f>MAX(D2:D4)</f>
+        <v>2400</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>